<commit_message>
ajout dde l'option filtre dans la vue éditeur
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Applications/MAMP/htdocs/php-mariadb-Questionary/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ahmed Tidjani\Documents\php-mariadb-Questionary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{64E2D9BA-920F-D94D-A216-B10991F67E0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{560EE083-8CE6-42FA-B718-5D1F768E8CE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Réponses" sheetId="2" r:id="rId1"/>
@@ -21,6 +21,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="d/m/yy\ h:mm;@"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -208,7 +211,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
@@ -240,20 +243,20 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{251AB61D-DB1C-0247-A16E-BA67D5AE47BF}"/>
   </cellStyles>
   <dxfs count="4">
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -273,6 +276,14 @@
     <dxf>
       <fill>
         <patternFill patternType="darkUp">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <fgColor rgb="FFFFFFFF"/>
           <bgColor rgb="FFFFFFFF"/>
         </patternFill>
@@ -624,71 +635,71 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5B48F7C-98C7-1247-B78D-EF5A1A340F47}">
   <sheetPr codeName="Feuil1"/>
   <dimension ref="A1:BE2571"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.1640625" style="19" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.5" style="2" customWidth="1"/>
+    <col min="1" max="1" width="15.109375" style="19" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" style="28" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.44140625" style="2" customWidth="1"/>
     <col min="4" max="4" width="26" style="2" customWidth="1"/>
-    <col min="5" max="5" width="27.5" style="2" customWidth="1"/>
+    <col min="5" max="5" width="27.44140625" style="2" customWidth="1"/>
     <col min="6" max="6" width="22.6640625" style="4" customWidth="1"/>
     <col min="7" max="7" width="25.6640625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="27.5" style="3" customWidth="1"/>
-    <col min="9" max="9" width="29.1640625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="27.44140625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="29.109375" style="2" customWidth="1"/>
     <col min="10" max="10" width="26" style="2" customWidth="1"/>
-    <col min="11" max="11" width="27.5" style="2" customWidth="1"/>
+    <col min="11" max="11" width="27.44140625" style="2" customWidth="1"/>
     <col min="12" max="12" width="22.6640625" style="4" customWidth="1"/>
     <col min="13" max="13" width="25.6640625" style="2" customWidth="1"/>
-    <col min="14" max="14" width="27.5" style="3" customWidth="1"/>
-    <col min="15" max="15" width="29.1640625" style="2" customWidth="1"/>
+    <col min="14" max="14" width="27.44140625" style="3" customWidth="1"/>
+    <col min="15" max="15" width="29.109375" style="2" customWidth="1"/>
     <col min="16" max="16" width="26" style="2" customWidth="1"/>
-    <col min="17" max="17" width="27.5" style="2" customWidth="1"/>
+    <col min="17" max="17" width="27.44140625" style="2" customWidth="1"/>
     <col min="18" max="18" width="22.6640625" style="4" customWidth="1"/>
     <col min="19" max="19" width="25.6640625" style="2" customWidth="1"/>
-    <col min="20" max="20" width="27.5" style="3" customWidth="1"/>
-    <col min="21" max="21" width="29.1640625" style="2" customWidth="1"/>
+    <col min="20" max="20" width="27.44140625" style="3" customWidth="1"/>
+    <col min="21" max="21" width="29.109375" style="2" customWidth="1"/>
     <col min="22" max="22" width="26" style="2" customWidth="1"/>
-    <col min="23" max="23" width="27.5" style="2" customWidth="1"/>
+    <col min="23" max="23" width="27.44140625" style="2" customWidth="1"/>
     <col min="24" max="24" width="22.6640625" style="4" customWidth="1"/>
     <col min="25" max="25" width="25.6640625" style="2" customWidth="1"/>
-    <col min="26" max="26" width="27.5" style="3" customWidth="1"/>
-    <col min="27" max="27" width="29.1640625" style="2" customWidth="1"/>
+    <col min="26" max="26" width="27.44140625" style="3" customWidth="1"/>
+    <col min="27" max="27" width="29.109375" style="2" customWidth="1"/>
     <col min="28" max="28" width="26" style="2" customWidth="1"/>
-    <col min="29" max="29" width="27.5" style="2" customWidth="1"/>
+    <col min="29" max="29" width="27.44140625" style="2" customWidth="1"/>
     <col min="30" max="30" width="22.6640625" style="4" customWidth="1"/>
     <col min="31" max="31" width="25.6640625" style="2" customWidth="1"/>
-    <col min="32" max="32" width="27.5" style="3" customWidth="1"/>
-    <col min="33" max="33" width="29.1640625" style="2" customWidth="1"/>
+    <col min="32" max="32" width="27.44140625" style="3" customWidth="1"/>
+    <col min="33" max="33" width="29.109375" style="2" customWidth="1"/>
     <col min="34" max="34" width="26" style="2" customWidth="1"/>
-    <col min="35" max="35" width="27.5" style="2" customWidth="1"/>
+    <col min="35" max="35" width="27.44140625" style="2" customWidth="1"/>
     <col min="36" max="36" width="22.6640625" style="4" customWidth="1"/>
     <col min="37" max="37" width="25.6640625" style="2" customWidth="1"/>
-    <col min="38" max="38" width="27.5" style="3" customWidth="1"/>
-    <col min="39" max="39" width="29.1640625" style="2" customWidth="1"/>
+    <col min="38" max="38" width="27.44140625" style="3" customWidth="1"/>
+    <col min="39" max="39" width="29.109375" style="2" customWidth="1"/>
     <col min="40" max="40" width="26" style="2" customWidth="1"/>
-    <col min="41" max="41" width="27.5" style="2" customWidth="1"/>
+    <col min="41" max="41" width="27.44140625" style="2" customWidth="1"/>
     <col min="42" max="42" width="22.6640625" style="4" customWidth="1"/>
     <col min="43" max="43" width="25.6640625" style="2" customWidth="1"/>
-    <col min="44" max="44" width="27.5" style="3" customWidth="1"/>
-    <col min="45" max="45" width="29.1640625" style="2" customWidth="1"/>
+    <col min="44" max="44" width="27.44140625" style="3" customWidth="1"/>
+    <col min="45" max="45" width="29.109375" style="2" customWidth="1"/>
     <col min="46" max="46" width="26" style="2" customWidth="1"/>
-    <col min="47" max="47" width="27.5" style="2" customWidth="1"/>
+    <col min="47" max="47" width="27.44140625" style="2" customWidth="1"/>
     <col min="48" max="48" width="22.6640625" style="4" customWidth="1"/>
     <col min="49" max="49" width="25.6640625" style="2" customWidth="1"/>
-    <col min="50" max="50" width="27.5" style="3" customWidth="1"/>
-    <col min="51" max="51" width="29.1640625" style="2" customWidth="1"/>
+    <col min="50" max="50" width="27.44140625" style="3" customWidth="1"/>
+    <col min="51" max="51" width="29.109375" style="2" customWidth="1"/>
     <col min="52" max="52" width="26" style="2" customWidth="1"/>
-    <col min="53" max="53" width="27.5" style="2" customWidth="1"/>
+    <col min="53" max="53" width="27.44140625" style="2" customWidth="1"/>
     <col min="54" max="54" width="22.6640625" style="4" customWidth="1"/>
     <col min="55" max="55" width="25.6640625" style="2" customWidth="1"/>
-    <col min="56" max="56" width="27.5" style="3" customWidth="1"/>
-    <col min="57" max="57" width="29.1640625" style="2" customWidth="1"/>
-    <col min="58" max="16384" width="8.83203125" style="1"/>
+    <col min="56" max="56" width="27.44140625" style="3" customWidth="1"/>
+    <col min="57" max="57" width="29.109375" style="2" customWidth="1"/>
+    <col min="58" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:57" x14ac:dyDescent="0.3">
       <c r="A1" s="17"/>
-      <c r="B1" s="17"/>
+      <c r="B1" s="23"/>
       <c r="C1" s="17"/>
       <c r="D1" s="17"/>
       <c r="E1" s="17"/>
@@ -745,9 +756,9 @@
       <c r="BD1" s="17"/>
       <c r="BE1" s="17"/>
     </row>
-    <row r="2" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:57" x14ac:dyDescent="0.3">
       <c r="A2" s="17"/>
-      <c r="B2" s="17"/>
+      <c r="B2" s="23"/>
       <c r="C2" s="17"/>
       <c r="D2" s="17"/>
       <c r="E2" s="17"/>
@@ -804,9 +815,9 @@
       <c r="BD2" s="17"/>
       <c r="BE2" s="17"/>
     </row>
-    <row r="3" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:57" x14ac:dyDescent="0.3">
       <c r="A3" s="17"/>
-      <c r="B3" s="17"/>
+      <c r="B3" s="23"/>
       <c r="C3" s="17"/>
       <c r="D3" s="17"/>
       <c r="E3" s="17"/>
@@ -863,9 +874,9 @@
       <c r="BD3" s="17"/>
       <c r="BE3" s="17"/>
     </row>
-    <row r="4" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:57" x14ac:dyDescent="0.3">
       <c r="A4" s="17"/>
-      <c r="B4" s="17"/>
+      <c r="B4" s="23"/>
       <c r="C4" s="17"/>
       <c r="D4" s="17"/>
       <c r="E4" s="17"/>
@@ -922,9 +933,9 @@
       <c r="BD4" s="17"/>
       <c r="BE4" s="17"/>
     </row>
-    <row r="5" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:57" x14ac:dyDescent="0.3">
       <c r="A5" s="17"/>
-      <c r="B5" s="17"/>
+      <c r="B5" s="23"/>
       <c r="C5" s="17"/>
       <c r="D5" s="17"/>
       <c r="E5" s="17"/>
@@ -981,9 +992,9 @@
       <c r="BD5" s="17"/>
       <c r="BE5" s="17"/>
     </row>
-    <row r="6" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:57" x14ac:dyDescent="0.3">
       <c r="A6" s="17"/>
-      <c r="B6" s="17"/>
+      <c r="B6" s="23"/>
       <c r="C6" s="17"/>
       <c r="D6" s="17"/>
       <c r="E6" s="17"/>
@@ -1040,9 +1051,9 @@
       <c r="BD6" s="17"/>
       <c r="BE6" s="17"/>
     </row>
-    <row r="7" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:57" x14ac:dyDescent="0.3">
       <c r="A7" s="17"/>
-      <c r="B7" s="17"/>
+      <c r="B7" s="23"/>
       <c r="C7" s="17"/>
       <c r="D7" s="17"/>
       <c r="E7" s="17"/>
@@ -1099,9 +1110,9 @@
       <c r="BD7" s="17"/>
       <c r="BE7" s="17"/>
     </row>
-    <row r="8" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:57" x14ac:dyDescent="0.3">
       <c r="A8" s="17"/>
-      <c r="B8" s="17"/>
+      <c r="B8" s="23"/>
       <c r="C8" s="17"/>
       <c r="D8" s="17"/>
       <c r="E8" s="17"/>
@@ -1158,9 +1169,9 @@
       <c r="BD8" s="17"/>
       <c r="BE8" s="17"/>
     </row>
-    <row r="9" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:57" x14ac:dyDescent="0.3">
       <c r="A9" s="17"/>
-      <c r="B9" s="17"/>
+      <c r="B9" s="23"/>
       <c r="C9" s="17"/>
       <c r="D9" s="17"/>
       <c r="E9" s="17"/>
@@ -1217,9 +1228,9 @@
       <c r="BD9" s="17"/>
       <c r="BE9" s="17"/>
     </row>
-    <row r="10" spans="1:57" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:57" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="16"/>
-      <c r="B10" s="14"/>
+      <c r="B10" s="24"/>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
       <c r="E10" s="14"/>
@@ -1276,9 +1287,9 @@
       <c r="BD10" s="15"/>
       <c r="BE10" s="14"/>
     </row>
-    <row r="11" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:57" x14ac:dyDescent="0.3">
       <c r="A11" s="18"/>
-      <c r="B11" s="11"/>
+      <c r="B11" s="25"/>
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
       <c r="E11" s="11"/>
@@ -1335,9 +1346,9 @@
       <c r="BD11" s="12"/>
       <c r="BE11" s="11"/>
     </row>
-    <row r="165" spans="1:57" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:57" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A165" s="20"/>
-      <c r="B165" s="8"/>
+      <c r="B165" s="26"/>
       <c r="C165" s="8"/>
       <c r="D165" s="8"/>
       <c r="E165" s="8"/>
@@ -1394,9 +1405,9 @@
       <c r="BD165" s="9"/>
       <c r="BE165" s="8"/>
     </row>
-    <row r="616" spans="1:57" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="616" spans="1:57" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A616" s="21"/>
-      <c r="B616" s="14"/>
+      <c r="B616" s="24"/>
       <c r="C616" s="14"/>
       <c r="D616" s="14"/>
       <c r="E616" s="14"/>
@@ -1453,9 +1464,9 @@
       <c r="BD616" s="15"/>
       <c r="BE616" s="14"/>
     </row>
-    <row r="617" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="617" spans="1:57" x14ac:dyDescent="0.3">
       <c r="A617" s="18"/>
-      <c r="B617" s="11"/>
+      <c r="B617" s="25"/>
       <c r="C617" s="11"/>
       <c r="D617" s="11"/>
       <c r="E617" s="11"/>
@@ -1512,9 +1523,9 @@
       <c r="BD617" s="12"/>
       <c r="BE617" s="11"/>
     </row>
-    <row r="771" spans="1:57" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="771" spans="1:57" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A771" s="20"/>
-      <c r="B771" s="8"/>
+      <c r="B771" s="26"/>
       <c r="C771" s="8"/>
       <c r="D771" s="8"/>
       <c r="E771" s="8"/>
@@ -1571,9 +1582,9 @@
       <c r="BD771" s="9"/>
       <c r="BE771" s="8"/>
     </row>
-    <row r="1222" spans="1:57" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1222" spans="1:57" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1222" s="21"/>
-      <c r="B1222" s="14"/>
+      <c r="B1222" s="24"/>
       <c r="C1222" s="14"/>
       <c r="D1222" s="14"/>
       <c r="E1222" s="14"/>
@@ -1630,9 +1641,9 @@
       <c r="BD1222" s="15"/>
       <c r="BE1222" s="14"/>
     </row>
-    <row r="1223" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="1223" spans="1:57" x14ac:dyDescent="0.3">
       <c r="A1223" s="18"/>
-      <c r="B1223" s="11"/>
+      <c r="B1223" s="25"/>
       <c r="C1223" s="11"/>
       <c r="D1223" s="11"/>
       <c r="E1223" s="11"/>
@@ -1689,9 +1700,9 @@
       <c r="BD1223" s="12"/>
       <c r="BE1223" s="11"/>
     </row>
-    <row r="1377" spans="1:57" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1377" spans="1:57" ht="16.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1377" s="20"/>
-      <c r="B1377" s="8"/>
+      <c r="B1377" s="26"/>
       <c r="C1377" s="8"/>
       <c r="D1377" s="8"/>
       <c r="E1377" s="8"/>
@@ -1748,9 +1759,9 @@
       <c r="BD1377" s="9"/>
       <c r="BE1377" s="8"/>
     </row>
-    <row r="2571" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="2571" spans="1:57" x14ac:dyDescent="0.3">
       <c r="A2571" s="22"/>
-      <c r="B2571" s="5"/>
+      <c r="B2571" s="27"/>
       <c r="C2571" s="5"/>
       <c r="D2571" s="5"/>
       <c r="E2571" s="5"/>
@@ -1808,29 +1819,29 @@
       <c r="BE2571" s="5"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A10:AX1464">
+    <cfRule type="containsBlanks" dxfId="3" priority="5">
+      <formula>NBCAR(SUPPRESPACE(A10))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A10:CA1693">
-    <cfRule type="containsBlanks" dxfId="3" priority="1">
-      <formula>_xludf.NBCAR(_xludf.SUPPRESPACE(A10))=0</formula>
+    <cfRule type="containsBlanks" dxfId="2" priority="1">
+      <formula>NBCAR(SUPPRESPACE(A10))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A10:CS1509">
-    <cfRule type="containsBlanks" dxfId="2" priority="2">
-      <formula>_xludf.NBCAR(_xludf.SUPPRESPACE(A10))=0</formula>
+    <cfRule type="containsBlanks" dxfId="1" priority="2">
+      <formula>NBCAR(SUPPRESPACE(A10))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A10:CT1698">
+    <cfRule type="containsBlanks" dxfId="0" priority="4">
+      <formula>NBCAR(SUPPRESPACE(A10))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D10:BE1509">
     <cfRule type="containsBlanks" priority="3">
-      <formula>_xludf.NBCAR(_xludf.SUPPRESPACE(D10))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A10:CT1698">
-    <cfRule type="containsBlanks" dxfId="1" priority="4">
-      <formula>_xludf.NBCAR(_xludf.SUPPRESPACE(A10))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A10:AX1464">
-    <cfRule type="containsBlanks" dxfId="0" priority="5">
-      <formula>_xludf.NBCAR(_xludf.SUPPRESPACE(A10))=0</formula>
+      <formula>NBCAR(SUPPRESPACE(D10))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>